<commit_message>
Update Short Semester I (E23 Batch).xlsx
</commit_message>
<xml_diff>
--- a/Short Semester I (E23 Batch).xlsx
+++ b/Short Semester I (E23 Batch).xlsx
@@ -1,16 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30131"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://uoj-my.sharepoint.com/personal/mayooran_eng_jfn_ac_lk/Documents/Short_Semesters/app/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\maids.jfn\Documents\GitHub\MC3020_Attendance\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="7" documentId="8_{1271330B-46C0-46A4-ACC4-A2400220E94A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8650D420-E038-4BBB-B8AB-CED52E4C9493}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="3"/>
   </bookViews>
   <sheets>
     <sheet name="MC9010" sheetId="2" r:id="rId1"/>
@@ -22,12 +21,12 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'MC9010'!$A$1:$F$170</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'MC9020'!$A$1:$F$111</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'MC9100'!$A$1:$G$189</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'MC9100'!$A$1:$G$190</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'MC9160'!$A$1:$H$172</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="3">'MC9100'!$1:$1</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="4">'MC9160'!#REF!</definedName>
   </definedNames>
-  <calcPr calcId="152511"/>
+  <calcPr calcId="152511" concurrentCalc="0"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -37,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1556" uniqueCount="572">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1557" uniqueCount="573">
   <si>
     <t>No.</t>
   </si>
@@ -1753,12 +1752,15 @@
   </si>
   <si>
     <t>BANDARANAYAKE K.M.R.D.</t>
+  </si>
+  <si>
+    <t>2021/E/033</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <fonts count="26" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -2175,7 +2177,7 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyBorder="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="88">
+  <cellXfs count="89">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -2424,13 +2426,16 @@
     <xf numFmtId="0" fontId="12" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="49" fontId="21" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="5">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Normal 15" xfId="2" xr:uid="{00000000-0005-0000-0000-000001000000}"/>
-    <cellStyle name="Normal 2" xfId="3" xr:uid="{00000000-0005-0000-0000-000002000000}"/>
-    <cellStyle name="Normal 2 2" xfId="4" xr:uid="{00000000-0005-0000-0000-000003000000}"/>
-    <cellStyle name="Normal_Sheet1" xfId="1" xr:uid="{00000000-0005-0000-0000-000004000000}"/>
+    <cellStyle name="Normal 15" xfId="2"/>
+    <cellStyle name="Normal 2" xfId="3"/>
+    <cellStyle name="Normal 2 2" xfId="4"/>
+    <cellStyle name="Normal_Sheet1" xfId="1"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -2711,7 +2716,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:G170"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -6303,7 +6308,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5E4A1C7F-0F69-4789-A5FA-AC8F6F6D4A56}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:G150"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -8991,7 +8996,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:G111"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.3"/>
   <cols>
@@ -11345,8 +11350,8 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:H189"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:H190"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="6.7109375" customWidth="1"/>
@@ -15801,68 +15806,58 @@
       <c r="H185" s="58"/>
     </row>
     <row r="186" spans="1:8" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A186" s="22">
-        <v>185</v>
-      </c>
-      <c r="B186" s="16" t="s">
-        <v>557</v>
-      </c>
-      <c r="C186" s="20" t="s">
-        <v>342</v>
-      </c>
-      <c r="D186" s="18">
-        <v>88</v>
-      </c>
+      <c r="A186" s="22"/>
+      <c r="B186" s="16"/>
+      <c r="C186" s="88" t="s">
+        <v>572</v>
+      </c>
+      <c r="D186" s="18"/>
       <c r="E186" s="18">
-        <v>67</v>
-      </c>
-      <c r="F186" s="18">
-        <v>75</v>
-      </c>
-      <c r="G186" s="53">
-        <v>62</v>
-      </c>
+        <v>77</v>
+      </c>
+      <c r="F186" s="18"/>
+      <c r="G186" s="53"/>
       <c r="H186" s="58"/>
     </row>
     <row r="187" spans="1:8" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A187" s="22">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="B187" s="16" t="s">
-        <v>472</v>
+        <v>557</v>
       </c>
       <c r="C187" s="20" t="s">
-        <v>343</v>
+        <v>342</v>
       </c>
       <c r="D187" s="18">
         <v>88</v>
       </c>
       <c r="E187" s="18">
-        <v>77</v>
+        <v>67</v>
       </c>
       <c r="F187" s="18">
         <v>75</v>
       </c>
       <c r="G187" s="53">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="H187" s="58"/>
     </row>
     <row r="188" spans="1:8" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A188" s="22">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="B188" s="16" t="s">
-        <v>473</v>
+        <v>472</v>
       </c>
       <c r="C188" s="20" t="s">
-        <v>344</v>
+        <v>343</v>
       </c>
       <c r="D188" s="18">
         <v>88</v>
       </c>
       <c r="E188" s="18">
-        <v>87</v>
+        <v>77</v>
       </c>
       <c r="F188" s="18">
         <v>75</v>
@@ -15872,29 +15867,53 @@
       </c>
       <c r="H188" s="58"/>
     </row>
-    <row r="189" spans="1:8" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A189" s="23">
+    <row r="189" spans="1:8" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A189" s="22">
+        <v>187</v>
+      </c>
+      <c r="B189" s="16" t="s">
+        <v>473</v>
+      </c>
+      <c r="C189" s="20" t="s">
+        <v>344</v>
+      </c>
+      <c r="D189" s="18">
+        <v>88</v>
+      </c>
+      <c r="E189" s="18">
+        <v>87</v>
+      </c>
+      <c r="F189" s="18">
+        <v>75</v>
+      </c>
+      <c r="G189" s="53">
+        <v>61</v>
+      </c>
+      <c r="H189" s="58"/>
+    </row>
+    <row r="190" spans="1:8" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A190" s="23">
         <v>188</v>
       </c>
-      <c r="B189" s="24" t="s">
+      <c r="B190" s="24" t="s">
         <v>558</v>
       </c>
-      <c r="C189" s="25" t="s">
+      <c r="C190" s="25" t="s">
         <v>345</v>
       </c>
-      <c r="D189" s="26">
+      <c r="D190" s="26">
         <v>88</v>
       </c>
-      <c r="E189" s="26">
-        <v>70</v>
-      </c>
-      <c r="F189" s="26">
-        <v>75</v>
-      </c>
-      <c r="G189" s="54">
+      <c r="E190" s="26">
+        <v>70</v>
+      </c>
+      <c r="F190" s="26">
+        <v>75</v>
+      </c>
+      <c r="G190" s="54">
         <v>64</v>
       </c>
-      <c r="H189" s="59"/>
+      <c r="H190" s="59"/>
     </row>
   </sheetData>
   <printOptions horizontalCentered="1"/>
@@ -15904,7 +15923,7 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:I168"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -20459,15 +20478,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <lcf76f155ced4ddcb4097134ff3c332f xmlns="2835d969-06cc-46e6-b4cc-c525f784ce43">
@@ -20478,7 +20488,7 @@
 </p:properties>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100455C4072EA7E0D46870C67AD0D3E62C3" ma:contentTypeVersion="18" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="6d62d4992a7888825600c982e6c75641">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="2835d969-06cc-46e6-b4cc-c525f784ce43" xmlns:ns3="03c84e3c-1549-479a-8619-e0d964aa7481" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="9015832621b6abd41b87bce5adc31c29" ns2:_="" ns3:_="">
     <xsd:import namespace="2835d969-06cc-46e6-b4cc-c525f784ce43"/>
@@ -20733,15 +20743,16 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{781D7AC4-6CC5-4242-91F0-BEE6E1ED618F}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CA8EACE5-8C5B-48FA-AFAD-2C86FB600767}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
@@ -20758,7 +20769,7 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{46A244EB-A970-4F2B-8B12-6A24EFA3E1AE}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -20775,4 +20786,12 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{781D7AC4-6CC5-4242-91F0-BEE6E1ED618F}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>